<commit_message>
Update Week 6 AI
</commit_message>
<xml_diff>
--- a/AI Audit Log_HoHuynhMinhHuy.xlsx
+++ b/AI Audit Log_HoHuynhMinhHuy.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="19392" windowHeight="11472" activeTab="4"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="19392" windowHeight="11472" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Week 1" sheetId="1" r:id="rId1"/>
@@ -17,6 +17,7 @@
     <sheet name="Week 3" sheetId="3" r:id="rId3"/>
     <sheet name="Week 4" sheetId="4" r:id="rId4"/>
     <sheet name="Week5" sheetId="5" r:id="rId5"/>
+    <sheet name="Week6" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="118">
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
@@ -325,6 +326,78 @@
   </si>
   <si>
     <t>Phản hồi: AI đề xuất sử dụng middleware xử lý lỗi tập trung và chuẩn hóa thông báo lỗi trả về client. Quyết định: Tôi xây dựng middleware riêng để quản lý lỗi và giảm trùng lặp code trong controller.</t>
+  </si>
+  <si>
+    <t>MongoDB Schema Design</t>
+  </si>
+  <si>
+    <t>"Thiết kế schema MongoDB cho hệ thống quản lý lịch hẹn bác sĩ gồm Doctor, Appointment và Patient."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất sử dụng ObjectId để liên kết dữ liệu và thiết kế các collection theo hướng chuẩn hóa. Quyết định: Tôi áp dụng mô hình tham chiếu dữ liệu bằng ObjectId và sử dụng populate để hiển thị thông tin liên quan.</t>
+  </si>
+  <si>
+    <t>Controller Development</t>
+  </si>
+  <si>
+    <t>"Giải thích chi tiết Appointment Controller sử dụng async/await trong NodeJS."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích luồng xử lý request, cách hoạt động của async/await và xử lý lỗi bằng try-catch. Quyết định: Tôi hiểu rõ hơn về bất đồng bộ trong JavaScript và cải thiện khả năng giải thích source code khi bảo vệ đồ án.</t>
+  </si>
+  <si>
+    <t>Business Logic Validation</t>
+  </si>
+  <si>
+    <t>"Kiểm tra logic tránh tạo nhiều phiên gửi xe cùng lúc cho một bãi đỗ."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất kiểm tra trạng thái slot trước khi tạo Parking Session mới và cập nhật trạng thái khi kết thúc phiên gửi xe. Quyết định: Tôi bổ sung điều kiện kiểm tra dữ liệu để tránh phát sinh dữ liệu không hợp lệ.</t>
+  </si>
+  <si>
+    <t>Prompt Engineering</t>
+  </si>
+  <si>
+    <t>"Viết prompt chi tiết để AI tạo ứng dụng Todo List bằng React Native theo mô hình component."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI xây dựng prompt mô tả đầy đủ cấu trúc thư mục, chức năng và giao diện. Quyết định: Tôi sử dụng prompt này để tăng hiệu quả hỗ trợ lập trình từ AI và tiết kiệm thời gian phát triển.</t>
+  </si>
+  <si>
+    <t>UI/UX Review</t>
+  </si>
+  <si>
+    <t>"Đánh giá giao diện hiện tại và đề xuất cải tiến để ứng dụng trông chuyên nghiệp hơn."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI chỉ ra các vấn đề về khoảng cách, màu sắc và bố cục, đồng thời đề xuất thiết kế hiện đại hơn. Quyết định: Tôi chỉnh sửa giao diện theo hướng tối giản và đồng nhất trải nghiệm người dùng.</t>
+  </si>
+  <si>
+    <t>Learning Support</t>
+  </si>
+  <si>
+    <t>"Giải thích chi tiết kiểm định Welch's t-test và ý nghĩa các công thức thống kê."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích từng bước suy luận, công thức và điều kiện áp dụng của phép kiểm định. Quyết định: Tôi sử dụng phần giải thích này để hiểu bản chất bài học thay vì chỉ ghi nhớ công thức.</t>
+  </si>
+  <si>
+    <t>Cloud Deployment</t>
+  </si>
+  <si>
+    <t>"Hướng dẫn deploy ứng dụng NodeJS lên Heroku và kết nối MongoDB Atlas."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI hướng dẫn cấu hình biến môi trường, Procfile, build script và cách whitelist IP trên MongoDB Atlas. Quyết định: Tôi thực hiện deploy thành công ứng dụng lên môi trường cloud và hiểu rõ quy trình triển khai thực tế.</t>
+  </si>
+  <si>
+    <t>REST API Development</t>
+  </si>
+  <si>
+    <t>"Xây dựng chức năng Create Booking với Mongoose và kiểm tra số lượng ghế còn trống."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI hướng dẫn validate dữ liệu đầu vào, cập nhật số ghế còn lại và sử dụng populate để lấy thông tin liên quan. Quyết định: Tôi áp dụng giải pháp vào bài thực hành SDN302 và hoàn thiện API đặt vé.</t>
   </si>
 </sst>
 </file>
@@ -1337,4 +1410,147 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
+  <cols>
+    <col min="1" max="1" width="20.8984375" customWidth="1"/>
+    <col min="2" max="2" width="26.8984375" customWidth="1"/>
+    <col min="3" max="3" width="25.19921875" customWidth="1"/>
+    <col min="4" max="4" width="52.296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="55.2">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="55.2">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="55.2">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="55.2">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="55.2">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="55.2">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="55.2">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="55.2">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>